<commit_message>
Batch 20 shipped: 5404N -06 thread fix + 4 long nipples (1,629 of 2,535)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04_DESIGN_TABLES/DesignTable_5404N.xlsx
+++ b/04_DESIGN_TABLES/DesignTable_5404N.xlsx
@@ -2030,14 +2030,37 @@
           <t>5404-N-06X4.500</t>
         </is>
       </c>
+      <c r="B29" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.675</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.675</v>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>5404-N-06X4.500</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>3/8-18 x 3/8-18 NPTF, cut length 4.5 in</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2047,7 +2070,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source</t>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | 2026-10-21 (batch 20): L from the part number, bar dia and bores from the Air-Way nipple 5404-N-06-06-X1 (A4 yes 2026-10-18), as every 06 sibling row; MISSING -&gt; ASSUMED</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2187,14 +2210,37 @@
           <t>5404-N-08X2.500</t>
         </is>
       </c>
+      <c r="B32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.84</v>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>5404-N-08X2.500</t>
         </is>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1/2-14 x 1/2-14 NPTF, cut length 2.5 in</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2204,7 +2250,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source</t>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | 2026-10-21 (batch 20): L from the part number, bar dia and bores from the Air-Way nipple 5404-N-08-08-X3 (A4 yes 2026-10-18), as every 08 sibling row; MISSING -&gt; ASSUMED</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2404,14 +2450,37 @@
           <t>5404-N-08X5.500</t>
         </is>
       </c>
+      <c r="B36" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.84</v>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>5404-N-08X5.500</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>1/2-14 x 1/2-14 NPTF, cut length 5.5 in</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2421,7 +2490,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source</t>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | 2026-10-21 (batch 20): L from the part number, bar dia and bores from the Air-Way nipple 5404-N-08-08-X3 (A4 yes 2026-10-18), as every 08 sibling row; MISSING -&gt; ASSUMED</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2531,7 +2600,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2541,7 +2610,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-10-18 (wave 3 adapters, staged, not shipped): NEW row - OMi sells this part (SKU dropped by the 2026-09-23 crawl; two-pass crawl 2026-10-16, tools/_out/adapters77_20261016/REPORT_77.md); Air-Way does not print this size; L from the part number, bar dia and bores from the Air-Way nipple 5404-N-06-06-X1 (A4 yes 2026-10-18); no Brennan size used</t>
+          <t>2026-10-18 (wave 3 adapters, staged, not shipped): NEW row - OMi sells this part (SKU dropped by the 2026-09-23 crawl; two-pass crawl 2026-10-16, tools/_out/adapters77_20261016/REPORT_77.md); Air-Way does not print this size; L from the part number, bar dia and bores from the Air-Way nipple 5404-N-06-06-X1 (A4 yes 2026-10-18); no Brennan size used | 2026-10-21 (batch 20): L from the part number, bar dia and bores from the Air-Way nipple 5404-N-06-06-X1 (A4 yes 2026-10-18), as every 06 sibling row; MISSING -&gt; ASSUMED</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">

</xml_diff>